<commit_message>
Salwar names, construction worker payment
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Sep26.xlsx
+++ b/docs/Chiraath-Summary-Sep26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{981932A2-332F-5849-87C8-D2712785B7AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66E4BE83-2814-4547-B274-C644FA88F445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">INVENTORY!$A$1:$T$272</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Purchases!$A$1:$D$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Sales!$A$1:$I$329</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Sales!$A$1:$I$334</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3551" uniqueCount="1398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3555" uniqueCount="1402">
   <si>
     <t>Notes:</t>
   </si>
@@ -3880,9 +3880,6 @@
     <t>Prajisha (Construction Company)</t>
   </si>
   <si>
-    <t>CHR-87 Red Salwar with Elephant print, CHR-58 Wine Red Salwar, CHR-180 Coffee Brown Salwar(M) (2100 advance, 1350 balance)</t>
-  </si>
-  <si>
     <t>Shinoob School - 1500(XXL), Niroop - XL, Prajisha(1100) - M</t>
   </si>
   <si>
@@ -3988,31 +3985,19 @@
     <t>Peacock blue/Royal blue, Purple/Pink, Lime Green/Wine Purple</t>
   </si>
   <si>
-    <t>426363 Churidar Set</t>
-  </si>
-  <si>
     <t>L, XL, XXL</t>
   </si>
   <si>
     <t>CHR-251</t>
   </si>
   <si>
-    <t>425677 Churidar Set</t>
-  </si>
-  <si>
     <t>M, L, XL, XXL</t>
   </si>
   <si>
     <t>CHR-252</t>
   </si>
   <si>
-    <t>417278 Churidar Set</t>
-  </si>
-  <si>
     <t>CHR-253</t>
-  </si>
-  <si>
-    <t>424938 Churidar Set</t>
   </si>
   <si>
     <t>Soft Silk Saree Collection (Kuthanpully)</t>
@@ -4257,6 +4242,33 @@
   </si>
   <si>
     <t>Mauve Purple, Deep Red / Maroon</t>
+  </si>
+  <si>
+    <t>425677 Churidar Set - Cotton Salwar 3 piece set</t>
+  </si>
+  <si>
+    <t>417278 Churidar Set - Chanderi Salwar 3 piece set</t>
+  </si>
+  <si>
+    <t>424938 Churidar Set - Silk Salwar 3 piece set</t>
+  </si>
+  <si>
+    <t>Navy Blue</t>
+  </si>
+  <si>
+    <t>CHR-87 Red Salwar with Elephant print, CHR-58 Wine Red Salwar, CHR-180 Coffee Brown Salwar(M) (3100 advance, 350 balance)</t>
+  </si>
+  <si>
+    <t>Olive gold</t>
+  </si>
+  <si>
+    <t>426363 Churidar Set - Chanderi Salwar multicolor flora set</t>
+  </si>
+  <si>
+    <t>Dusty Rose</t>
+  </si>
+  <si>
+    <t>Chocolate Brown.</t>
   </si>
 </sst>
 </file>
@@ -6099,13 +6111,13 @@
                   <c:v>72915</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>65156</c:v>
+                  <c:v>66256</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>79098</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>8860</c:v>
+                  <c:v>8960</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -6539,13 +6551,13 @@
                   <c:v>-26128</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-37044</c:v>
+                  <c:v>-35944</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>33250</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>17052</c:v>
+                  <c:v>17152</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -8213,7 +8225,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>568331</v>
+        <v>568431</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -8230,7 +8242,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>581411</v>
+        <v>582611</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -8247,7 +8259,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-25672</v>
+        <v>-25572</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -8463,11 +8475,11 @@
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>189481.55539999998</v>
+        <v>189514.89539999998</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>306196.44460000005</v>
+        <v>306163.10460000002</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -8475,11 +8487,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>168886.41860000003</v>
+        <v>168853.07860000001</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹168,886</v>
+        <v>Pay ₹168,853</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -8489,15 +8501,15 @@
       </c>
       <c r="B27" s="12">
         <f>'Cash Pool'!B5</f>
-        <v>59123</v>
+        <v>59223</v>
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>189367.88920000001</v>
+        <v>189401.20920000001</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-130244.88920000001</v>
+        <v>-130178.20920000001</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -8505,11 +8517,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-58657.847200000004</v>
+        <v>-58591.167200000011</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹58,658</v>
+        <v>Receive ₹58,591</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -8523,11 +8535,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>189481.55539999998</v>
+        <v>189514.89539999998</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-176951.55539999998</v>
+        <v>-176984.89539999998</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -8535,11 +8547,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-111228.57139999997</v>
+        <v>-111261.91139999997</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹111,229</v>
+        <v>Receive ₹111,262</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -8651,7 +8663,7 @@
       </c>
       <c r="B3" s="20">
         <f ca="1">TODAY()</f>
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -8667,7 +8679,7 @@
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>568331</v>
+        <v>568431</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -8676,7 +8688,7 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-25672</v>
+        <v>-25572</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
@@ -8840,11 +8852,11 @@
       </c>
       <c r="C16" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$993,"MMM")=$A16)*(YEAR(Sales!$A$2:$A$993)=$B$7)*Sales!$C$2:$C$993),0)</f>
-        <v>65156</v>
+        <v>66256</v>
       </c>
       <c r="D16" s="21">
         <f t="shared" si="0"/>
-        <v>-37044</v>
+        <v>-35944</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" customHeight="1">
@@ -8874,11 +8886,11 @@
       </c>
       <c r="C18" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$993,"MMM")=$A18)*(YEAR(Sales!$A$2:$A$993)=$B$7)*Sales!$C$2:$C$993),0)</f>
-        <v>8860</v>
+        <v>8960</v>
       </c>
       <c r="D18" s="21">
         <f t="shared" si="0"/>
-        <v>17052</v>
+        <v>17152</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15" customHeight="1">
@@ -10625,7 +10637,7 @@
         <v>3046</v>
       </c>
       <c r="D110" s="36" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="111" spans="1:4" ht="15" customHeight="1">
@@ -10695,7 +10707,7 @@
         <v>-4202</v>
       </c>
       <c r="D115" s="39" t="s">
-        <v>1388</v>
+        <v>1383</v>
       </c>
     </row>
     <row r="116" spans="1:4" ht="15" customHeight="1">
@@ -10709,7 +10721,7 @@
         <v>-1620</v>
       </c>
       <c r="D116" s="36" t="s">
-        <v>1388</v>
+        <v>1383</v>
       </c>
     </row>
     <row r="117" spans="1:4" ht="15" customHeight="1">
@@ -10723,7 +10735,7 @@
         <v>-603</v>
       </c>
       <c r="D117" s="39" t="s">
-        <v>1388</v>
+        <v>1383</v>
       </c>
     </row>
     <row r="118" spans="1:4" ht="15" customHeight="1">
@@ -10737,7 +10749,7 @@
         <v>-1911</v>
       </c>
       <c r="D118" s="36" t="s">
-        <v>1388</v>
+        <v>1383</v>
       </c>
     </row>
     <row r="119" spans="1:4" ht="15" customHeight="1">
@@ -19281,7 +19293,7 @@
       <c r="F265" s="46"/>
       <c r="G265" s="46"/>
       <c r="H265" s="46" t="s">
-        <v>1367</v>
+        <v>1362</v>
       </c>
       <c r="I265" s="45" t="s">
         <v>148</v>
@@ -19345,14 +19357,14 @@
         <v>1271</v>
       </c>
       <c r="C268" s="83">
-        <v>2350</v>
+        <v>3450</v>
       </c>
       <c r="D268" s="44"/>
       <c r="E268" s="44"/>
       <c r="F268" s="44"/>
       <c r="G268" s="44"/>
       <c r="H268" s="44" t="s">
-        <v>1272</v>
+        <v>1397</v>
       </c>
       <c r="I268" s="44" t="s">
         <v>356</v>
@@ -19388,7 +19400,7 @@
         <v>46210</v>
       </c>
       <c r="B270" s="44" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
       <c r="C270" s="83">
         <v>3200</v>
@@ -19663,7 +19675,7 @@
         <v>46219</v>
       </c>
       <c r="B281" s="45" t="s">
-        <v>1329</v>
+        <v>1324</v>
       </c>
       <c r="C281" s="85">
         <v>3600</v>
@@ -19677,7 +19689,7 @@
       <c r="F281" s="46"/>
       <c r="G281" s="46"/>
       <c r="H281" s="46" t="s">
-        <v>1331</v>
+        <v>1326</v>
       </c>
       <c r="I281" s="45" t="s">
         <v>148</v>
@@ -19938,7 +19950,7 @@
         <v>46229</v>
       </c>
       <c r="B292" s="45" t="s">
-        <v>1369</v>
+        <v>1364</v>
       </c>
       <c r="C292" s="85">
         <v>3600</v>
@@ -19948,7 +19960,7 @@
       <c r="F292" s="46"/>
       <c r="G292" s="46"/>
       <c r="H292" s="46" t="s">
-        <v>1368</v>
+        <v>1363</v>
       </c>
       <c r="I292" s="45" t="s">
         <v>356</v>
@@ -19969,7 +19981,7 @@
       <c r="F293" s="44"/>
       <c r="G293" s="44"/>
       <c r="H293" s="44" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
       <c r="I293" s="44" t="s">
         <v>356</v>
@@ -19994,7 +20006,7 @@
       <c r="F294" s="46"/>
       <c r="G294" s="46"/>
       <c r="H294" s="46" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
       <c r="I294" s="45" t="s">
         <v>148</v>
@@ -20055,7 +20067,7 @@
         <v>46236</v>
       </c>
       <c r="B297" s="44" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
       <c r="C297" s="83">
         <v>6900</v>
@@ -20069,7 +20081,7 @@
       <c r="F297" s="44"/>
       <c r="G297" s="44"/>
       <c r="H297" s="44" t="s">
-        <v>1276</v>
+        <v>1275</v>
       </c>
       <c r="I297" s="44" t="s">
         <v>148</v>
@@ -20155,7 +20167,7 @@
         <v>46238</v>
       </c>
       <c r="B301" s="44" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
       <c r="C301" s="83">
         <v>12650</v>
@@ -20169,7 +20181,7 @@
       <c r="F301" s="44"/>
       <c r="G301" s="44"/>
       <c r="H301" s="44" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="I301" s="44" t="s">
         <v>148</v>
@@ -20215,7 +20227,7 @@
       <c r="F303" s="44"/>
       <c r="G303" s="44"/>
       <c r="H303" s="44" t="s">
-        <v>1372</v>
+        <v>1367</v>
       </c>
       <c r="I303" s="44" t="s">
         <v>148</v>
@@ -20240,7 +20252,7 @@
       <c r="F304" s="46"/>
       <c r="G304" s="46"/>
       <c r="H304" s="46" t="s">
-        <v>1366</v>
+        <v>1361</v>
       </c>
       <c r="I304" s="45" t="s">
         <v>148</v>
@@ -20301,7 +20313,7 @@
         <v>46243</v>
       </c>
       <c r="B307" s="44" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
       <c r="C307" s="83">
         <v>5750</v>
@@ -20315,7 +20327,7 @@
       <c r="F307" s="44"/>
       <c r="G307" s="44"/>
       <c r="H307" s="44" t="s">
-        <v>1275</v>
+        <v>1274</v>
       </c>
       <c r="I307" s="44" t="s">
         <v>148</v>
@@ -20451,7 +20463,7 @@
         <v>46252</v>
       </c>
       <c r="B313" s="45" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
       <c r="C313" s="85">
         <v>5750</v>
@@ -20465,7 +20477,7 @@
       <c r="F313" s="46"/>
       <c r="G313" s="46"/>
       <c r="H313" s="46" t="s">
-        <v>1275</v>
+        <v>1274</v>
       </c>
       <c r="I313" s="45" t="s">
         <v>148</v>
@@ -20476,7 +20488,7 @@
         <v>46252</v>
       </c>
       <c r="B314" s="44" t="s">
-        <v>1278</v>
+        <v>1277</v>
       </c>
       <c r="C314" s="83">
         <v>1380</v>
@@ -20490,7 +20502,7 @@
       <c r="F314" s="44"/>
       <c r="G314" s="44"/>
       <c r="H314" s="44" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="I314" s="44" t="s">
         <v>148</v>
@@ -20501,7 +20513,7 @@
         <v>46252</v>
       </c>
       <c r="B315" s="45" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
       <c r="C315" s="85">
         <v>5750</v>
@@ -20515,7 +20527,7 @@
       <c r="F315" s="46"/>
       <c r="G315" s="46"/>
       <c r="H315" s="46" t="s">
-        <v>1275</v>
+        <v>1274</v>
       </c>
       <c r="I315" s="45" t="s">
         <v>148</v>
@@ -20526,7 +20538,7 @@
         <v>46252</v>
       </c>
       <c r="B316" s="44" t="s">
-        <v>1282</v>
+        <v>1281</v>
       </c>
       <c r="C316" s="83">
         <v>1340</v>
@@ -20540,7 +20552,7 @@
       <c r="F316" s="44"/>
       <c r="G316" s="44"/>
       <c r="H316" s="44" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
       <c r="I316" s="44" t="s">
         <v>148</v>
@@ -20551,7 +20563,7 @@
         <v>46252</v>
       </c>
       <c r="B317" s="45" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
       <c r="C317" s="85">
         <v>1250</v>
@@ -20565,7 +20577,7 @@
       <c r="F317" s="46"/>
       <c r="G317" s="46"/>
       <c r="H317" s="46" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="I317" s="45" t="s">
         <v>148</v>
@@ -20576,7 +20588,7 @@
         <v>46257</v>
       </c>
       <c r="B318" s="44" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
       <c r="C318" s="83">
         <v>1780</v>
@@ -20590,7 +20602,7 @@
       <c r="F318" s="44"/>
       <c r="G318" s="44"/>
       <c r="H318" s="44" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="I318" s="44" t="s">
         <v>148</v>
@@ -20615,7 +20627,7 @@
       <c r="F319" s="46"/>
       <c r="G319" s="46"/>
       <c r="H319" s="46" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="I319" s="45" t="s">
         <v>148</v>
@@ -20640,7 +20652,7 @@
       <c r="F320" s="44"/>
       <c r="G320" s="44"/>
       <c r="H320" s="44" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
       <c r="I320" s="44" t="s">
         <v>148</v>
@@ -20651,7 +20663,7 @@
         <v>46257</v>
       </c>
       <c r="B321" s="45" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="C321" s="85">
         <v>1500</v>
@@ -20665,7 +20677,7 @@
       <c r="F321" s="46"/>
       <c r="G321" s="46"/>
       <c r="H321" s="46" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="I321" s="45" t="s">
         <v>148</v>
@@ -20676,7 +20688,7 @@
         <v>46258</v>
       </c>
       <c r="B322" s="44" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="C322" s="83">
         <v>1250</v>
@@ -20690,7 +20702,7 @@
       <c r="F322" s="44"/>
       <c r="G322" s="44"/>
       <c r="H322" s="44" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="I322" s="44" t="s">
         <v>148</v>
@@ -20701,7 +20713,7 @@
         <v>46263</v>
       </c>
       <c r="B323" s="45" t="s">
-        <v>1320</v>
+        <v>1315</v>
       </c>
       <c r="C323" s="85">
         <v>1380</v>
@@ -20715,7 +20727,7 @@
       <c r="F323" s="46"/>
       <c r="G323" s="46"/>
       <c r="H323" s="46" t="s">
-        <v>1321</v>
+        <v>1316</v>
       </c>
       <c r="I323" s="45" t="s">
         <v>148</v>
@@ -20726,7 +20738,7 @@
         <v>46263</v>
       </c>
       <c r="B324" s="44" t="s">
-        <v>1323</v>
+        <v>1318</v>
       </c>
       <c r="C324" s="83">
         <v>1380</v>
@@ -20740,7 +20752,7 @@
       <c r="F324" s="44"/>
       <c r="G324" s="44"/>
       <c r="H324" s="44" t="s">
-        <v>1324</v>
+        <v>1319</v>
       </c>
       <c r="I324" s="44" t="s">
         <v>148</v>
@@ -20751,7 +20763,7 @@
         <v>46263</v>
       </c>
       <c r="B325" s="45" t="s">
-        <v>1325</v>
+        <v>1320</v>
       </c>
       <c r="C325" s="85">
         <v>2500</v>
@@ -20765,7 +20777,7 @@
       <c r="F325" s="46"/>
       <c r="G325" s="46"/>
       <c r="H325" s="46" t="s">
-        <v>1335</v>
+        <v>1330</v>
       </c>
       <c r="I325" s="45" t="s">
         <v>148</v>
@@ -20790,7 +20802,7 @@
       <c r="F326" s="44"/>
       <c r="G326" s="44"/>
       <c r="H326" s="44" t="s">
-        <v>1334</v>
+        <v>1329</v>
       </c>
       <c r="I326" s="44" t="s">
         <v>148</v>
@@ -20801,7 +20813,7 @@
         <v>46257</v>
       </c>
       <c r="B327" s="45" t="s">
-        <v>1336</v>
+        <v>1331</v>
       </c>
       <c r="C327" s="85">
         <v>750</v>
@@ -20815,7 +20827,7 @@
       <c r="F327" s="46"/>
       <c r="G327" s="46"/>
       <c r="H327" s="46" t="s">
-        <v>1337</v>
+        <v>1332</v>
       </c>
       <c r="I327" s="45" t="s">
         <v>148</v>
@@ -20826,7 +20838,7 @@
         <v>46275</v>
       </c>
       <c r="B328" s="44" t="s">
-        <v>1373</v>
+        <v>1368</v>
       </c>
       <c r="C328" s="83">
         <v>1380</v>
@@ -20840,7 +20852,7 @@
       <c r="F328" s="44"/>
       <c r="G328" s="44"/>
       <c r="H328" s="44" t="s">
-        <v>1374</v>
+        <v>1369</v>
       </c>
       <c r="I328" s="44" t="s">
         <v>148</v>
@@ -20861,7 +20873,7 @@
       <c r="F329" s="46"/>
       <c r="G329" s="46"/>
       <c r="H329" s="46" t="s">
-        <v>1375</v>
+        <v>1370</v>
       </c>
       <c r="I329" s="45" t="s">
         <v>356</v>
@@ -20872,7 +20884,7 @@
         <v>46275</v>
       </c>
       <c r="B330" s="44" t="s">
-        <v>1377</v>
+        <v>1372</v>
       </c>
       <c r="C330" s="83">
         <v>1450</v>
@@ -20886,7 +20898,7 @@
       <c r="F330" s="44"/>
       <c r="G330" s="44"/>
       <c r="H330" s="44" t="s">
-        <v>1380</v>
+        <v>1375</v>
       </c>
       <c r="I330" s="44" t="s">
         <v>148</v>
@@ -20897,7 +20909,7 @@
         <v>46275</v>
       </c>
       <c r="B331" s="45" t="s">
-        <v>1384</v>
+        <v>1379</v>
       </c>
       <c r="C331" s="85">
         <v>950</v>
@@ -20911,7 +20923,7 @@
       <c r="F331" s="46"/>
       <c r="G331" s="46"/>
       <c r="H331" s="46" t="s">
-        <v>1385</v>
+        <v>1380</v>
       </c>
       <c r="I331" s="45" t="s">
         <v>148</v>
@@ -20936,7 +20948,7 @@
       <c r="F332" s="44"/>
       <c r="G332" s="44"/>
       <c r="H332" s="44" t="s">
-        <v>1393</v>
+        <v>1388</v>
       </c>
       <c r="I332" s="44" t="s">
         <v>148</v>
@@ -20950,7 +20962,7 @@
         <v>183</v>
       </c>
       <c r="C333" s="85">
-        <v>650</v>
+        <v>750</v>
       </c>
       <c r="D333" s="45" t="s">
         <v>150</v>
@@ -20961,7 +20973,7 @@
       <c r="F333" s="46"/>
       <c r="G333" s="46"/>
       <c r="H333" s="46" t="s">
-        <v>1394</v>
+        <v>1389</v>
       </c>
       <c r="I333" s="45" t="s">
         <v>148</v>
@@ -20978,7 +20990,7 @@
         <v>1380</v>
       </c>
       <c r="D334" s="44" t="s">
-        <v>1395</v>
+        <v>1390</v>
       </c>
       <c r="E334" s="44" t="s">
         <v>49</v>
@@ -20986,7 +20998,7 @@
       <c r="F334" s="44"/>
       <c r="G334" s="44"/>
       <c r="H334" s="44" t="s">
-        <v>1374</v>
+        <v>1369</v>
       </c>
       <c r="I334" s="44" t="s">
         <v>148</v>
@@ -21202,7 +21214,7 @@
       <c r="I353" s="45"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I329" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <autoFilter ref="A1:I334" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1257" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>"Ordered,Pending,Completed,Cancelled"</formula1>
@@ -21234,7 +21246,7 @@
     <col min="13" max="13" width="22.5" style="47" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="11.83203125" style="47" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="14.6640625" style="47" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="62.6640625" style="47" customWidth="1"/>
+    <col min="16" max="16" width="62" style="47" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="14.83203125" style="47" customWidth="1"/>
     <col min="18" max="18" width="11.1640625" style="47" customWidth="1"/>
     <col min="19" max="20" width="10" style="48" customWidth="1"/>
@@ -28835,7 +28847,7 @@
         <v>0</v>
       </c>
       <c r="L78" s="52" t="s">
-        <v>1381</v>
+        <v>1376</v>
       </c>
       <c r="M78" s="52"/>
       <c r="N78" s="52" t="s">
@@ -29155,14 +29167,14 @@
         <v>450</v>
       </c>
       <c r="L84" s="52" t="s">
-        <v>1379</v>
+        <v>1374</v>
       </c>
       <c r="M84" s="52"/>
       <c r="N84" s="52" t="s">
         <v>589</v>
       </c>
       <c r="O84" s="52" t="s">
-        <v>1378</v>
+        <v>1373</v>
       </c>
       <c r="P84" s="52"/>
       <c r="Q84" s="52"/>
@@ -29261,14 +29273,14 @@
         <v>1045</v>
       </c>
       <c r="L86" s="52" t="s">
-        <v>1382</v>
+        <v>1377</v>
       </c>
       <c r="M86" s="52"/>
       <c r="N86" s="52" t="s">
         <v>589</v>
       </c>
       <c r="O86" s="52" t="s">
-        <v>1383</v>
+        <v>1378</v>
       </c>
       <c r="P86" s="52"/>
       <c r="Q86" s="52"/>
@@ -31075,7 +31087,7 @@
       </c>
       <c r="O120" s="52"/>
       <c r="P120" s="52" t="s">
-        <v>1346</v>
+        <v>1341</v>
       </c>
       <c r="Q120" s="52"/>
       <c r="R120" s="52"/>
@@ -34163,7 +34175,7 @@
         <v>606</v>
       </c>
       <c r="L166" s="52" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
       <c r="M166" s="52"/>
       <c r="N166" s="52" t="s">
@@ -34171,7 +34183,7 @@
       </c>
       <c r="O166" s="52"/>
       <c r="P166" s="52" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="Q166" s="52"/>
       <c r="R166" s="52"/>
@@ -34959,7 +34971,7 @@
         <v>1019</v>
       </c>
       <c r="L181" s="55" t="s">
-        <v>1273</v>
+        <v>1272</v>
       </c>
       <c r="M181" s="55"/>
       <c r="N181" s="55" t="s">
@@ -35272,7 +35284,7 @@
         <v>891</v>
       </c>
       <c r="L187" s="55" t="s">
-        <v>1278</v>
+        <v>1277</v>
       </c>
       <c r="M187" s="55"/>
       <c r="N187" s="55" t="s">
@@ -35376,7 +35388,7 @@
         <v>891</v>
       </c>
       <c r="L189" s="55" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
       <c r="M189" s="55"/>
       <c r="N189" s="55" t="s">
@@ -35384,7 +35396,7 @@
       </c>
       <c r="O189" s="55"/>
       <c r="P189" s="55" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
       <c r="Q189" s="55"/>
       <c r="R189" s="55"/>
@@ -35627,14 +35639,14 @@
         <v>3950</v>
       </c>
       <c r="L194" s="52" t="s">
-        <v>1328</v>
+        <v>1323</v>
       </c>
       <c r="M194" s="52"/>
       <c r="N194" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P194" s="47" t="s">
-        <v>1386</v>
+        <v>1381</v>
       </c>
       <c r="S194" s="47"/>
       <c r="T194" s="47"/>
@@ -35827,14 +35839,14 @@
         <v>934</v>
       </c>
       <c r="L198" s="55" t="s">
-        <v>1391</v>
+        <v>1386</v>
       </c>
       <c r="M198" s="55"/>
       <c r="N198" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P198" s="47" t="s">
-        <v>1390</v>
+        <v>1385</v>
       </c>
       <c r="S198" s="47"/>
       <c r="T198" s="47"/>
@@ -35878,14 +35890,14 @@
         <v>1732</v>
       </c>
       <c r="L199" s="52" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
       <c r="M199" s="52"/>
       <c r="N199" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P199" s="47" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
       <c r="S199" s="47"/>
       <c r="T199" s="47"/>
@@ -35946,7 +35958,7 @@
         <v>996</v>
       </c>
       <c r="B201" s="55" t="s">
-        <v>1371</v>
+        <v>1366</v>
       </c>
       <c r="C201" s="55" t="s">
         <v>95</v>
@@ -35987,7 +35999,7 @@
         <v>589</v>
       </c>
       <c r="P201" s="47" t="s">
-        <v>1370</v>
+        <v>1365</v>
       </c>
       <c r="S201" s="47"/>
       <c r="T201" s="47"/>
@@ -36133,7 +36145,7 @@
         <v>0</v>
       </c>
       <c r="L204" s="55" t="s">
-        <v>1392</v>
+        <v>1387</v>
       </c>
       <c r="M204" s="55"/>
       <c r="N204" s="47" t="s">
@@ -36283,14 +36295,14 @@
         <v>2346</v>
       </c>
       <c r="L207" s="52" t="s">
-        <v>1327</v>
+        <v>1322</v>
       </c>
       <c r="M207" s="52"/>
       <c r="N207" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P207" s="47" t="s">
-        <v>1326</v>
+        <v>1321</v>
       </c>
       <c r="S207" s="47"/>
       <c r="T207" s="47"/>
@@ -36434,7 +36446,7 @@
         <v>0</v>
       </c>
       <c r="L210" s="55" t="s">
-        <v>1332</v>
+        <v>1327</v>
       </c>
       <c r="M210" s="55"/>
       <c r="N210" s="47" t="s">
@@ -36485,7 +36497,7 @@
         <v>0</v>
       </c>
       <c r="L211" s="52" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
       <c r="M211" s="52"/>
       <c r="N211" s="47" t="s">
@@ -36533,14 +36545,14 @@
         <v>2775</v>
       </c>
       <c r="L212" s="55" t="s">
-        <v>1387</v>
+        <v>1382</v>
       </c>
       <c r="M212" s="55"/>
       <c r="N212" s="47" t="s">
         <v>504</v>
       </c>
       <c r="P212" s="47" t="s">
-        <v>1330</v>
+        <v>1325</v>
       </c>
       <c r="S212" s="47"/>
       <c r="T212" s="47"/>
@@ -36584,7 +36596,7 @@
         <v>3340</v>
       </c>
       <c r="L213" s="52" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="M213" s="52"/>
       <c r="N213" s="47" t="s">
@@ -36837,7 +36849,7 @@
         <v>761</v>
       </c>
       <c r="L218" s="55" t="s">
-        <v>1376</v>
+        <v>1371</v>
       </c>
       <c r="M218" s="55"/>
       <c r="N218" s="47" t="s">
@@ -37339,7 +37351,7 @@
         <v>0</v>
       </c>
       <c r="L228" s="52" t="s">
-        <v>1364</v>
+        <v>1359</v>
       </c>
       <c r="M228" s="52"/>
       <c r="N228" s="47" t="s">
@@ -37641,14 +37653,14 @@
         <v>1824</v>
       </c>
       <c r="L234" s="52" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="M234" s="52"/>
       <c r="N234" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P234" s="86" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
       <c r="S234" s="47"/>
       <c r="T234" s="47"/>
@@ -37692,7 +37704,7 @@
         <v>734</v>
       </c>
       <c r="L235" s="55" t="s">
-        <v>1365</v>
+        <v>1360</v>
       </c>
       <c r="M235" s="55"/>
       <c r="N235" s="47" t="s">
@@ -37848,7 +37860,7 @@
         <v>677</v>
       </c>
       <c r="P238" s="86" t="s">
-        <v>1389</v>
+        <v>1384</v>
       </c>
       <c r="S238" s="47"/>
       <c r="T238" s="47"/>
@@ -38045,7 +38057,7 @@
         <v>0</v>
       </c>
       <c r="L242" s="52" t="s">
-        <v>1333</v>
+        <v>1328</v>
       </c>
       <c r="M242" s="52"/>
       <c r="N242" s="47" t="s">
@@ -38753,7 +38765,7 @@
         <v>1223</v>
       </c>
       <c r="B248" s="52" t="s">
-        <v>1317</v>
+        <v>1312</v>
       </c>
       <c r="C248" s="52" t="s">
         <v>95</v>
@@ -38792,17 +38804,17 @@
         <v>677</v>
       </c>
       <c r="P248" s="86" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="S248" s="47"/>
       <c r="T248" s="47"/>
     </row>
     <row r="249" spans="1:246" ht="17">
       <c r="A249" s="55" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
       <c r="B249" s="55" t="s">
-        <v>1318</v>
+        <v>1313</v>
       </c>
       <c r="C249" s="55" t="s">
         <v>95</v>
@@ -38841,17 +38853,17 @@
         <v>677</v>
       </c>
       <c r="P249" s="86" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="S249" s="47"/>
       <c r="T249" s="47"/>
     </row>
-    <row r="250" spans="1:246" ht="16">
+    <row r="250" spans="1:246" ht="17">
       <c r="A250" s="52" t="s">
-        <v>1305</v>
+        <v>1304</v>
       </c>
       <c r="B250" s="52" t="s">
-        <v>1308</v>
+        <v>1399</v>
       </c>
       <c r="C250" s="52" t="s">
         <v>96</v>
@@ -38859,7 +38871,9 @@
       <c r="D250" s="53">
         <v>1090</v>
       </c>
-      <c r="E250" s="53"/>
+      <c r="E250" s="53">
+        <v>1650</v>
+      </c>
       <c r="F250" s="66">
         <v>0</v>
       </c>
@@ -38888,18 +38902,20 @@
         <v>677</v>
       </c>
       <c r="O250" s="47" t="s">
-        <v>1309</v>
-      </c>
-      <c r="P250" s="86"/>
+        <v>1307</v>
+      </c>
+      <c r="P250" s="86" t="s">
+        <v>1401</v>
+      </c>
       <c r="S250" s="47"/>
       <c r="T250" s="47"/>
     </row>
-    <row r="251" spans="1:246" ht="16">
+    <row r="251" spans="1:246" ht="17">
       <c r="A251" s="55" t="s">
-        <v>1310</v>
+        <v>1308</v>
       </c>
       <c r="B251" s="55" t="s">
-        <v>1311</v>
+        <v>1393</v>
       </c>
       <c r="C251" s="55" t="s">
         <v>96</v>
@@ -38907,7 +38923,9 @@
       <c r="D251" s="56">
         <v>1049</v>
       </c>
-      <c r="E251" s="56"/>
+      <c r="E251" s="56">
+        <v>1550</v>
+      </c>
       <c r="F251" s="64">
         <v>0</v>
       </c>
@@ -38936,18 +38954,20 @@
         <v>677</v>
       </c>
       <c r="O251" s="47" t="s">
-        <v>1312</v>
-      </c>
-      <c r="P251" s="86"/>
+        <v>1309</v>
+      </c>
+      <c r="P251" s="86" t="s">
+        <v>1396</v>
+      </c>
       <c r="S251" s="47"/>
       <c r="T251" s="47"/>
     </row>
-    <row r="252" spans="1:246" ht="16">
+    <row r="252" spans="1:246" ht="17">
       <c r="A252" s="52" t="s">
-        <v>1313</v>
+        <v>1310</v>
       </c>
       <c r="B252" s="52" t="s">
-        <v>1314</v>
+        <v>1394</v>
       </c>
       <c r="C252" s="52" t="s">
         <v>96</v>
@@ -38955,7 +38975,9 @@
       <c r="D252" s="53">
         <v>1049</v>
       </c>
-      <c r="E252" s="53"/>
+      <c r="E252" s="53">
+        <v>1550</v>
+      </c>
       <c r="F252" s="66">
         <v>0</v>
       </c>
@@ -38984,18 +39006,20 @@
         <v>677</v>
       </c>
       <c r="O252" s="47" t="s">
-        <v>1312</v>
-      </c>
-      <c r="P252" s="86"/>
+        <v>1309</v>
+      </c>
+      <c r="P252" s="86" t="s">
+        <v>1398</v>
+      </c>
       <c r="S252" s="47"/>
       <c r="T252" s="47"/>
     </row>
-    <row r="253" spans="1:246" ht="16">
+    <row r="253" spans="1:246" ht="17">
       <c r="A253" s="55" t="s">
-        <v>1315</v>
+        <v>1311</v>
       </c>
       <c r="B253" s="55" t="s">
-        <v>1316</v>
+        <v>1395</v>
       </c>
       <c r="C253" s="55" t="s">
         <v>96</v>
@@ -39003,7 +39027,9 @@
       <c r="D253" s="56">
         <v>1322</v>
       </c>
-      <c r="E253" s="56"/>
+      <c r="E253" s="56">
+        <v>1900</v>
+      </c>
       <c r="F253" s="64">
         <v>0</v>
       </c>
@@ -39032,18 +39058,20 @@
         <v>677</v>
       </c>
       <c r="O253" s="47" t="s">
-        <v>1309</v>
-      </c>
-      <c r="P253" s="86"/>
+        <v>1307</v>
+      </c>
+      <c r="P253" s="86" t="s">
+        <v>1400</v>
+      </c>
       <c r="S253" s="47"/>
       <c r="T253" s="47"/>
     </row>
     <row r="254" spans="1:246" ht="16">
       <c r="A254" s="52" t="s">
-        <v>1319</v>
+        <v>1314</v>
       </c>
       <c r="B254" s="52" t="s">
-        <v>1341</v>
+        <v>1336</v>
       </c>
       <c r="C254" s="52" t="s">
         <v>95</v>
@@ -39077,7 +39105,7 @@
         <v>3564</v>
       </c>
       <c r="L254" s="52" t="s">
-        <v>1320</v>
+        <v>1315</v>
       </c>
       <c r="M254" s="52"/>
       <c r="N254" s="47" t="s">
@@ -39089,10 +39117,10 @@
     </row>
     <row r="255" spans="1:246" ht="16">
       <c r="A255" s="55" t="s">
-        <v>1322</v>
+        <v>1317</v>
       </c>
       <c r="B255" s="55" t="s">
-        <v>1342</v>
+        <v>1337</v>
       </c>
       <c r="C255" s="55" t="s">
         <v>95</v>
@@ -39126,7 +39154,7 @@
         <v>0</v>
       </c>
       <c r="L255" s="55" t="s">
-        <v>1396</v>
+        <v>1391</v>
       </c>
       <c r="M255" s="55"/>
       <c r="N255" s="47" t="s">
@@ -39138,10 +39166,10 @@
     </row>
     <row r="256" spans="1:246" ht="16">
       <c r="A256" s="52" t="s">
+        <v>1333</v>
+      </c>
+      <c r="B256" s="52" t="s">
         <v>1338</v>
-      </c>
-      <c r="B256" s="52" t="s">
-        <v>1343</v>
       </c>
       <c r="C256" s="52" t="s">
         <v>95</v>
@@ -39185,10 +39213,10 @@
     </row>
     <row r="257" spans="1:246" ht="16">
       <c r="A257" s="55" t="s">
+        <v>1334</v>
+      </c>
+      <c r="B257" s="55" t="s">
         <v>1339</v>
-      </c>
-      <c r="B257" s="55" t="s">
-        <v>1344</v>
       </c>
       <c r="C257" s="55" t="s">
         <v>95</v>
@@ -39232,10 +39260,10 @@
     </row>
     <row r="258" spans="1:246" ht="16">
       <c r="A258" s="52" t="s">
+        <v>1335</v>
+      </c>
+      <c r="B258" s="52" t="s">
         <v>1340</v>
-      </c>
-      <c r="B258" s="52" t="s">
-        <v>1345</v>
       </c>
       <c r="C258" s="52" t="s">
         <v>95</v>
@@ -39279,10 +39307,10 @@
     </row>
     <row r="259" spans="1:246" ht="17">
       <c r="A259" s="55" t="s">
-        <v>1347</v>
+        <v>1342</v>
       </c>
       <c r="B259" s="55" t="s">
-        <v>1358</v>
+        <v>1353</v>
       </c>
       <c r="C259" s="55" t="s">
         <v>95</v>
@@ -39321,17 +39349,17 @@
         <v>677</v>
       </c>
       <c r="P259" s="86" t="s">
-        <v>1359</v>
+        <v>1354</v>
       </c>
       <c r="S259" s="47"/>
       <c r="T259" s="47"/>
     </row>
     <row r="260" spans="1:246" ht="17">
       <c r="A260" s="52" t="s">
-        <v>1348</v>
+        <v>1343</v>
       </c>
       <c r="B260" s="52" t="s">
-        <v>1360</v>
+        <v>1355</v>
       </c>
       <c r="C260" s="52" t="s">
         <v>95</v>
@@ -39370,17 +39398,17 @@
         <v>677</v>
       </c>
       <c r="P260" s="86" t="s">
-        <v>1363</v>
+        <v>1358</v>
       </c>
       <c r="S260" s="47"/>
       <c r="T260" s="47"/>
     </row>
     <row r="261" spans="1:246" ht="17">
       <c r="A261" s="55" t="s">
+        <v>1344</v>
+      </c>
+      <c r="B261" s="55" t="s">
         <v>1349</v>
-      </c>
-      <c r="B261" s="55" t="s">
-        <v>1354</v>
       </c>
       <c r="C261" s="55" t="s">
         <v>95</v>
@@ -39419,17 +39447,17 @@
         <v>677</v>
       </c>
       <c r="P261" s="86" t="s">
-        <v>1355</v>
+        <v>1350</v>
       </c>
       <c r="S261" s="47"/>
       <c r="T261" s="47"/>
     </row>
     <row r="262" spans="1:246" ht="17">
       <c r="A262" s="52" t="s">
-        <v>1350</v>
+        <v>1345</v>
       </c>
       <c r="B262" s="52" t="s">
-        <v>1353</v>
+        <v>1348</v>
       </c>
       <c r="C262" s="52" t="s">
         <v>95</v>
@@ -39468,17 +39496,17 @@
         <v>677</v>
       </c>
       <c r="P262" s="86" t="s">
-        <v>1397</v>
+        <v>1392</v>
       </c>
       <c r="S262" s="47"/>
       <c r="T262" s="47"/>
     </row>
     <row r="263" spans="1:246" s="62" customFormat="1" ht="17">
       <c r="A263" s="87" t="s">
+        <v>1346</v>
+      </c>
+      <c r="B263" s="87" t="s">
         <v>1351</v>
-      </c>
-      <c r="B263" s="87" t="s">
-        <v>1356</v>
       </c>
       <c r="C263" s="87" t="s">
         <v>95</v>
@@ -39517,7 +39545,7 @@
         <v>677</v>
       </c>
       <c r="P263" s="91" t="s">
-        <v>1357</v>
+        <v>1352</v>
       </c>
       <c r="U263" s="61"/>
       <c r="V263" s="61"/>
@@ -39748,10 +39776,10 @@
     </row>
     <row r="264" spans="1:246" ht="34">
       <c r="A264" s="52" t="s">
-        <v>1352</v>
+        <v>1347</v>
       </c>
       <c r="B264" s="52" t="s">
-        <v>1361</v>
+        <v>1356</v>
       </c>
       <c r="C264" s="52" t="s">
         <v>95</v>
@@ -39790,7 +39818,7 @@
         <v>677</v>
       </c>
       <c r="P264" s="86" t="s">
-        <v>1362</v>
+        <v>1357</v>
       </c>
       <c r="S264" s="47"/>
       <c r="T264" s="47"/>
@@ -46196,11 +46224,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>189481.55539999998</v>
+        <v>189514.89539999998</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>306196.44460000005</v>
+        <v>306163.10460000002</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -46208,7 +46236,7 @@
       </c>
       <c r="G4" s="73">
         <f>E4+F4</f>
-        <v>168886.41860000003</v>
+        <v>168853.07860000001</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -46217,7 +46245,7 @@
       </c>
       <c r="B5" s="11">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A5,Sales!$I:$I,"Completed"),0)</f>
-        <v>59123</v>
+        <v>59223</v>
       </c>
       <c r="C5" s="11">
         <f>VLOOKUP($A5,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -46225,11 +46253,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>189367.88920000001</v>
+        <v>189401.20920000001</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-130244.88920000001</v>
+        <v>-130178.20920000001</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -46237,7 +46265,7 @@
       </c>
       <c r="G5" s="74">
         <f>E5+F5</f>
-        <v>-58657.847200000004</v>
+        <v>-58591.167200000011</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -46254,11 +46282,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>189481.55539999998</v>
+        <v>189514.89539999998</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-176951.55539999998</v>
+        <v>-176984.89539999998</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -46266,7 +46294,7 @@
       </c>
       <c r="G6" s="73">
         <f>E6+F6</f>
-        <v>-111228.57139999997</v>
+        <v>-111261.91139999997</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">

</xml_diff>